<commit_message>
Record hosted #18 final-closure evidence for Product Leadership review.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/private-beta/hosted-ux-qa/supreme-ai/Supreme-AI-Register.xlsx
+++ b/docs/private-beta/hosted-ux-qa/supreme-ai/Supreme-AI-Register.xlsx
@@ -34,10 +34,10 @@
     <t>Claims triage assistant</t>
   </si>
   <si>
-    <t>APPROVED</t>
-  </si>
-  <si>
-    <t>NOT_CLASSIFIED</t>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>Not Classified</t>
   </si>
   <si>
     <t>Unassigned</t>

</xml_diff>